<commit_message>
Fixed excel uploading issue
</commit_message>
<xml_diff>
--- a/Results/Actual_vs_estimated what if.xlsx
+++ b/Results/Actual_vs_estimated what if.xlsx
@@ -1431,598 +1431,598 @@
         </is>
       </c>
       <c r="B2" s="1" t="n">
-        <v>96.82025388583101</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>196980.8933511847</v>
+        <v>96.1002786080159</v>
+      </c>
+      <c r="C2" t="n">
+        <v>196233.3870365402</v>
       </c>
       <c r="D2" t="n">
-        <v>85.348357196384</v>
+        <v>84.81794728597005</v>
       </c>
       <c r="E2" t="n">
-        <v>28.87847580567497</v>
+        <v>29.86438052079079</v>
       </c>
       <c r="F2" t="n">
-        <v>842.6576944817438</v>
+        <v>842.2453125593397</v>
       </c>
       <c r="G2" t="n">
-        <v>57155.90000596788</v>
+        <v>57165.86959201389</v>
       </c>
       <c r="H2" s="1" t="n">
-        <v>31.66193253986926</v>
+        <v>32.52725823697558</v>
       </c>
       <c r="I2" t="n">
-        <v>4414.93494547526</v>
+        <v>4418.076291232639</v>
       </c>
       <c r="J2" s="1" t="n">
-        <v>240.3066491293765</v>
+        <v>239.4114282922831</v>
       </c>
       <c r="K2" t="n">
-        <v>7360.421487901475</v>
+        <v>7357.398166232639</v>
       </c>
       <c r="L2" s="1" t="n">
-        <v>3844.761407025595</v>
+        <v>3845.708012863409</v>
       </c>
       <c r="M2" t="n">
-        <v>14.59539912144924</v>
+        <v>14.37677280690959</v>
       </c>
       <c r="N2" t="n">
-        <v>16.09203407296015</v>
+        <v>16.03911888285955</v>
       </c>
       <c r="O2" t="n">
-        <v>18.83281043479749</v>
+        <v>19.04962718826735</v>
       </c>
       <c r="P2" t="n">
-        <v>0.7767959800008982</v>
+        <v>0.5108625211175107</v>
       </c>
       <c r="Q2" t="n">
-        <v>18.06662320988469</v>
+        <v>18.11625065970433</v>
       </c>
       <c r="R2" t="n">
-        <v>290.0101920628007</v>
+        <v>290.505781224843</v>
       </c>
       <c r="S2" t="n">
-        <v>17.96496948108193</v>
+        <v>18.01872530053965</v>
       </c>
       <c r="T2" t="n">
-        <v>18.29332903910259</v>
+        <v>18.3489091825872</v>
       </c>
       <c r="U2" t="n">
-        <v>16.83967696133872</v>
+        <v>16.85512170690792</v>
       </c>
       <c r="V2" t="n">
-        <v>17.5247924803824</v>
+        <v>17.47341171865489</v>
       </c>
       <c r="W2" t="n">
-        <v>15.95296551798561</v>
+        <v>16.11508476008023</v>
       </c>
       <c r="X2" t="n">
-        <v>16.78773636655666</v>
+        <v>16.98475526444523</v>
       </c>
       <c r="Y2" t="n">
-        <v>15.98698359184501</v>
+        <v>15.54201876632454</v>
       </c>
       <c r="Z2" t="n">
-        <v>304.8101953804814</v>
+        <v>304.6532722517559</v>
       </c>
       <c r="AA2" t="n">
-        <v>1400.470064425485</v>
+        <v>1399.712373522052</v>
       </c>
       <c r="AB2" t="n">
-        <v>40.57847796105802</v>
+        <v>41.32790663383762</v>
       </c>
       <c r="AC2" t="n">
-        <v>800.0132895526766</v>
+        <v>799.9708947734933</v>
       </c>
       <c r="AD2" t="n">
-        <v>32.18420081938228</v>
+        <v>33.00818938960315</v>
       </c>
       <c r="AE2" s="1" t="n">
-        <v>76.40748598680814</v>
+        <v>77.01000006001533</v>
       </c>
       <c r="AF2" t="n">
-        <v>18.27885269588894</v>
+        <v>18.3017648129993</v>
       </c>
       <c r="AG2" t="n">
-        <v>198.8416915534126</v>
+        <v>197.8452721434326</v>
       </c>
       <c r="AH2" t="n">
-        <v>32.11438748448063</v>
+        <v>33.01682885789435</v>
       </c>
       <c r="AI2" t="n">
-        <v>34.93451950544255</v>
+        <v>35.97283846120372</v>
       </c>
       <c r="AJ2" t="n">
-        <v>203.1754389562441</v>
+        <v>201.4590200196819</v>
       </c>
       <c r="AK2" t="n">
-        <v>38.21450648444897</v>
+        <v>39.42238512068942</v>
       </c>
       <c r="AL2" t="n">
-        <v>449.9652374565553</v>
+        <v>452.3300378615192</v>
       </c>
       <c r="AM2" t="n">
-        <v>43.22966687433099</v>
+        <v>44.63835280195035</v>
       </c>
       <c r="AN2" t="n">
-        <v>989.5489964092047</v>
+        <v>988.9359199155318</v>
       </c>
       <c r="AO2" t="n">
-        <v>34.67384935208698</v>
+        <v>35.73468394642134</v>
       </c>
       <c r="AP2" t="n">
-        <v>1940.473365190136</v>
+        <v>1942.713186013357</v>
       </c>
       <c r="AQ2" t="n">
-        <v>242.3854250084702</v>
+        <v>242.1755184848817</v>
       </c>
       <c r="AR2" t="n">
-        <v>539.7055492122339</v>
+        <v>540.1758146174237</v>
       </c>
       <c r="AS2" t="n">
-        <v>1082.995338322184</v>
+        <v>1085.27512636813</v>
       </c>
       <c r="AT2" t="n">
-        <v>1911.107010262186</v>
+        <v>1917.684187624319</v>
       </c>
       <c r="AU2" t="n">
-        <v>99.35952136447766</v>
+        <v>100.4576666896562</v>
       </c>
       <c r="AV2" t="n">
-        <v>99.60142093287085</v>
+        <v>100.8734312561504</v>
       </c>
       <c r="AW2" t="n">
-        <v>105.9512477144461</v>
+        <v>107.2501222944425</v>
       </c>
       <c r="AX2" t="n">
-        <v>106.3554835841655</v>
+        <v>107.6587302940672</v>
       </c>
       <c r="AY2" t="n">
-        <v>95.76843548764639</v>
+        <v>96.69519790135796</v>
       </c>
       <c r="AZ2" t="n">
-        <v>8468.952514860366</v>
+        <v>8450.902524736193</v>
       </c>
       <c r="BA2" t="n">
-        <v>8239.654965294732</v>
+        <v>8218.649270587497</v>
       </c>
       <c r="BB2" t="n">
-        <v>8550.24224556817</v>
+        <v>8502.252428690592</v>
       </c>
       <c r="BC2" t="n">
-        <v>7867.709108988443</v>
+        <v>7822.475045628018</v>
       </c>
       <c r="BD2" t="n">
-        <v>7788.446044286091</v>
+        <v>7750.848289065891</v>
       </c>
       <c r="BE2" s="1" t="n">
-        <v>468.8483085069687</v>
+        <v>470.0308203426312</v>
       </c>
       <c r="BF2" t="n">
-        <v>-36.84912678429915</v>
+        <v>-36.84574792509388</v>
       </c>
       <c r="BG2" s="2" t="n">
-        <v>25.85384955471096</v>
+        <v>25.68476407508645</v>
       </c>
       <c r="BH2" t="n">
-        <v>179.6068804054969</v>
+        <v>180.7269279439286</v>
       </c>
       <c r="BI2" s="1" t="n">
-        <v>261.3732381672667</v>
+        <v>257.7698002084406</v>
       </c>
       <c r="BJ2" t="n">
-        <v>-20.56177921977318</v>
+        <v>-20.42557869526833</v>
       </c>
       <c r="BK2" t="n">
-        <v>171.689271281081</v>
+        <v>172.5678298490173</v>
       </c>
       <c r="BL2" t="n">
-        <v>532.8288359305047</v>
+        <v>521.7768965371132</v>
       </c>
       <c r="BM2" t="n">
-        <v>222.5874488777051</v>
+        <v>221.2991761258517</v>
       </c>
       <c r="BN2" t="n">
-        <v>48.65824039357815</v>
+        <v>49.48784729625582</v>
       </c>
       <c r="BO2" t="n">
-        <v>609.0547884843229</v>
+        <v>625.9043125014481</v>
       </c>
       <c r="BP2" t="n">
-        <v>1989.268917603081</v>
+        <v>2044.925754646833</v>
       </c>
       <c r="BQ2" t="n">
-        <v>103.6756565138099</v>
+        <v>105.014509473473</v>
       </c>
       <c r="BR2" t="n">
-        <v>226.7164183246115</v>
+        <v>229.9418141614595</v>
       </c>
       <c r="BS2" t="n">
-        <v>165.9412706192992</v>
+        <v>167.563452187068</v>
       </c>
       <c r="BT2" t="n">
-        <v>87.61500399437786</v>
+        <v>88.63955924741153</v>
       </c>
       <c r="BU2" t="n">
-        <v>4430.608328781358</v>
+        <v>4433.798892840635</v>
       </c>
       <c r="BV2" t="n">
-        <v>418.9206057179052</v>
+        <v>420.3838762862646</v>
       </c>
       <c r="BW2" s="1" t="n">
-        <v>3676.349243164062</v>
+        <v>3684.537506103516</v>
       </c>
       <c r="BX2" t="n">
-        <v>2117.867764687487</v>
+        <v>2116.918537219165</v>
       </c>
       <c r="BY2" t="n">
-        <v>15.97011746205296</v>
+        <v>16.20303567418958</v>
       </c>
       <c r="BZ2" t="n">
-        <v>52.99210852931461</v>
+        <v>53.25350461204947</v>
       </c>
       <c r="CA2" t="n">
-        <v>2479.953762400643</v>
+        <v>2490.674168523923</v>
       </c>
       <c r="CB2" t="n">
-        <v>1094.704710728958</v>
+        <v>1124.53018701425</v>
       </c>
       <c r="CC2" s="1" t="n">
-        <v>0.7403163305483759</v>
+        <v>0.502452888712287</v>
       </c>
       <c r="CD2" t="n">
-        <v>2.250554752675661</v>
+        <v>2.317626868429789</v>
       </c>
       <c r="CE2" t="n">
-        <v>-144.9966100436181</v>
+        <v>-144.9974314231062</v>
       </c>
       <c r="CF2" t="n">
-        <v>9.134824586844086</v>
+        <v>9.040561654281364</v>
       </c>
       <c r="CG2" t="n">
-        <v>-13.83017876866687</v>
+        <v>-13.7299829115497</v>
       </c>
       <c r="CH2" t="n">
-        <v>9.118757133841113</v>
+        <v>8.973377293491325</v>
       </c>
       <c r="CI2" t="n">
-        <v>-69.710179551971</v>
+        <v>-70.7415158625839</v>
       </c>
       <c r="CJ2" t="n">
-        <v>269.7793363841042</v>
+        <v>269.0368456613842</v>
       </c>
       <c r="CK2" t="n">
-        <v>2644.156546467249</v>
+        <v>2635.112429772635</v>
       </c>
       <c r="CL2" t="n">
-        <v>8.983371692111021</v>
+        <v>9.566313228303008</v>
       </c>
       <c r="CM2" t="n">
-        <v>77.77902387024814</v>
+        <v>76.94437624441434</v>
       </c>
       <c r="CN2" t="n">
-        <v>307.7769802244029</v>
+        <v>304.4441176520172</v>
       </c>
       <c r="CO2" t="n">
-        <v>3239.354945903857</v>
+        <v>3239.655051078771</v>
       </c>
       <c r="CP2" t="n">
-        <v>139.4160564635893</v>
+        <v>151.4108453169872</v>
       </c>
       <c r="CQ2" t="n">
-        <v>33.30007171630859</v>
+        <v>35.30004119873047</v>
       </c>
       <c r="CR2" t="n">
-        <v>175.6883113368979</v>
+        <v>175.4719457056262</v>
       </c>
       <c r="CS2" t="n">
-        <v>7.503603818242921</v>
+        <v>6.896210396122391</v>
       </c>
       <c r="CT2" t="n">
-        <v>5.812239416312256</v>
+        <v>5.311792281538858</v>
       </c>
       <c r="CU2" t="n">
-        <v>0.05301481755962111</v>
+        <v>0.03754002849996621</v>
       </c>
       <c r="CV2" t="n">
-        <v>2991.585474560653</v>
+        <v>2997.409859566566</v>
       </c>
       <c r="CW2" t="n">
-        <v>0.1210366375138174</v>
+        <v>0.09224786285573815</v>
       </c>
       <c r="CX2" t="n">
-        <v>17.26905897589323</v>
+        <v>18.11900051196469</v>
       </c>
       <c r="CY2" t="n">
-        <v>68.94845319439881</v>
+        <v>68.51558768270841</v>
       </c>
       <c r="CZ2" t="n">
         <v>105</v>
       </c>
       <c r="DA2" t="n">
-        <v>88.35028269541391</v>
+        <v>88.32133820475433</v>
       </c>
       <c r="DB2" t="n">
-        <v>72.57378432612231</v>
+        <v>72.49572429306056</v>
       </c>
       <c r="DC2" t="n">
-        <v>3.66395998052945</v>
+        <v>3.833675112531711</v>
       </c>
       <c r="DD2" t="n">
-        <v>17.76116411358734</v>
+        <v>13.81361400176535</v>
       </c>
       <c r="DE2" t="n">
-        <v>67.99499879211103</v>
+        <v>67.93809728353015</v>
       </c>
       <c r="DF2" t="n">
-        <v>3262.605488067773</v>
+        <v>3261.86282984533</v>
       </c>
       <c r="DG2" t="n">
-        <v>524.9563487206626</v>
+        <v>525.0989262197851</v>
       </c>
       <c r="DH2" t="n">
-        <v>-95.40830102543691</v>
+        <v>-95.74228136284748</v>
       </c>
       <c r="DI2" t="n">
-        <v>4.636369243435272</v>
+        <v>4.199992977743014</v>
       </c>
       <c r="DJ2" t="n">
-        <v>2989.750536133151</v>
+        <v>2989.267244112629</v>
       </c>
       <c r="DK2" t="n">
-        <v>-116.7022297241444</v>
+        <v>-117.9165558463937</v>
       </c>
       <c r="DL2" t="n">
-        <v>750.0585303068567</v>
+        <v>754.9545954521207</v>
       </c>
       <c r="DM2" t="n">
-        <v>53.45445653792587</v>
+        <v>54.24999025412212</v>
       </c>
       <c r="DN2" t="n">
-        <v>-56.50688991125233</v>
+        <v>-41.4344737703999</v>
       </c>
       <c r="DO2" s="1" t="n">
-        <v>24.73292678470408</v>
+        <v>24.27128743560568</v>
       </c>
       <c r="DP2" t="n">
-        <v>-98.92852320659505</v>
-      </c>
-      <c r="DQ2" s="2" t="n">
-        <v>21.99230232678222</v>
+        <v>-99.39330338806586</v>
+      </c>
+      <c r="DQ2" s="1" t="n">
+        <v>16.30398306296808</v>
       </c>
       <c r="DR2" s="1" t="n">
-        <v>56.24413080962533</v>
+        <v>56.18535187038947</v>
       </c>
       <c r="DS2" t="n">
-        <v>-74.06344771666863</v>
+        <v>-74.54844866170986</v>
       </c>
       <c r="DT2" t="n">
-        <v>33.2337575810471</v>
+        <v>30.69948667154742</v>
       </c>
       <c r="DU2" t="n">
-        <v>79.62947714839412</v>
+        <v>80.756324054592</v>
       </c>
       <c r="DV2" t="n">
-        <v>-53.86953281720486</v>
+        <v>-54.12040356920902</v>
       </c>
       <c r="DW2" t="n">
-        <v>825.6840684151401</v>
+        <v>818.9290604379709</v>
       </c>
       <c r="DX2" t="n">
-        <v>3073.196516326414</v>
+        <v>3072.122124083681</v>
       </c>
       <c r="DY2" s="1" t="n">
-        <v>42.93755601902753</v>
+        <v>42.84441833621419</v>
       </c>
       <c r="DZ2" s="1" t="n">
-        <v>7531.606201171875</v>
+        <v>7564.690063476562</v>
       </c>
       <c r="EA2" t="n">
-        <v>11.15814744000261</v>
+        <v>11.61825760009534</v>
       </c>
       <c r="EB2" t="n">
-        <v>48.34009790449397</v>
+        <v>49.55690453660036</v>
       </c>
       <c r="EC2" t="n">
-        <v>1871.478120039137</v>
+        <v>1883.618344916694</v>
       </c>
       <c r="ED2" s="1" t="n">
-        <v>10190.77478027344</v>
+        <v>10110.21081542969</v>
       </c>
       <c r="EE2" t="n">
-        <v>0.8223883137106895</v>
-      </c>
-      <c r="EF2" s="1" t="n">
-        <v>127.1032033258289</v>
+        <v>0.8240583389997482</v>
+      </c>
+      <c r="EF2" t="n">
+        <v>126.452726754487</v>
       </c>
       <c r="EG2" t="n">
-        <v>95.98804975412475</v>
+        <v>95.97200523152152</v>
       </c>
       <c r="EH2" t="n">
-        <v>0.9459427649003515</v>
+        <v>0.9233596056824488</v>
       </c>
       <c r="EI2" t="n">
-        <v>97.6175555828557</v>
+        <v>97.63591734287353</v>
       </c>
       <c r="EJ2" t="n">
-        <v>0.9431872915084042</v>
+        <v>0.9114688517023549</v>
       </c>
       <c r="EK2" t="n">
-        <v>299.4201775347054</v>
+        <v>299.5135586775037</v>
       </c>
       <c r="EL2" s="1" t="n">
-        <v>40915.0048789978</v>
-      </c>
-      <c r="EM2" s="1" t="n">
-        <v>842.5824760277212</v>
+        <v>40745.12755870819</v>
+      </c>
+      <c r="EM2" s="2" t="n">
+        <v>842.4206308855208</v>
       </c>
       <c r="EN2" t="n">
-        <v>649.9187321924995</v>
+        <v>648.6757025004936</v>
       </c>
       <c r="EO2" t="n">
-        <v>50.33966254419578</v>
+        <v>52.58045898343432</v>
       </c>
       <c r="EP2" t="n">
-        <v>65.37802829695413</v>
+        <v>65.22768847430098</v>
       </c>
       <c r="EQ2" t="n">
-        <v>63.55928097471713</v>
+        <v>64.24428018058454</v>
       </c>
       <c r="ER2" t="n">
-        <v>0.2904927058694518</v>
+        <v>0.2918296852988182</v>
       </c>
       <c r="ES2" t="n">
-        <v>109.6573505417168</v>
+        <v>110.2921527896275</v>
       </c>
       <c r="ET2" t="n">
-        <v>78.16269866877332</v>
+        <v>79.82268863403179</v>
       </c>
       <c r="EU2" t="n">
-        <v>29.99961232125018</v>
-      </c>
-      <c r="EV2" s="1" t="n">
-        <v>423.5469548802906</v>
-      </c>
-      <c r="EW2" s="1" t="n">
-        <v>1300.48892532199</v>
-      </c>
-      <c r="EX2" s="1" t="n">
-        <v>5777.327410576188</v>
-      </c>
-      <c r="EY2" s="2" t="n">
-        <v>1.944566142542782</v>
+        <v>29.99832643704054</v>
+      </c>
+      <c r="EV2" t="n">
+        <v>424.1379562353861</v>
+      </c>
+      <c r="EW2" t="n">
+        <v>1301.51653599988</v>
+      </c>
+      <c r="EX2" t="n">
+        <v>5761.366241375794</v>
+      </c>
+      <c r="EY2" t="n">
+        <v>1.944692855491665</v>
       </c>
       <c r="EZ2" t="n">
-        <v>26.08518441139056</v>
-      </c>
-      <c r="FA2" s="1" t="n">
-        <v>1237.56463733229</v>
-      </c>
-      <c r="FB2" s="1" t="n">
-        <v>3.857237094226991</v>
+        <v>26.0723117842812</v>
+      </c>
+      <c r="FA2" t="n">
+        <v>1239.193944973814</v>
+      </c>
+      <c r="FB2" t="n">
+        <v>3.861328239384998</v>
       </c>
       <c r="FC2" t="n">
-        <v>98.10277213745483</v>
+        <v>98.16088491447424</v>
       </c>
       <c r="FD2" t="n">
-        <v>1.390217379490118</v>
+        <v>1.344008784731304</v>
       </c>
       <c r="FE2" t="n">
         <v>11</v>
       </c>
-      <c r="FF2" s="1" t="n">
-        <v>0.6383960569320176</v>
+      <c r="FF2" s="2" t="n">
+        <v>0.6377372248823373</v>
       </c>
       <c r="FG2" s="1" t="n">
-        <v>69.87769002535579</v>
-      </c>
-      <c r="FH2" s="2" t="n">
-        <v>35.47434923080346</v>
+        <v>69.78066028205319</v>
+      </c>
+      <c r="FH2" s="1" t="n">
+        <v>35.56003457712295</v>
       </c>
       <c r="FI2" s="2" t="n">
-        <v>2.803620174420379</v>
+        <v>2.799650600646601</v>
       </c>
       <c r="FJ2" s="1" t="n">
-        <v>167229.6100536866</v>
-      </c>
-      <c r="FK2" t="n">
-        <v>5.848705965880382</v>
+        <v>167889.1002448927</v>
+      </c>
+      <c r="FK2" s="1" t="n">
+        <v>5.865151487426161</v>
       </c>
       <c r="FL2" s="1" t="n">
-        <v>124851.8135351874</v>
-      </c>
-      <c r="FM2" s="2" t="n">
-        <v>12.17513464703528</v>
-      </c>
-      <c r="FN2" t="n">
-        <v>43763.69143976998</v>
+        <v>124088.9723157785</v>
+      </c>
+      <c r="FM2" s="1" t="n">
+        <v>12.45139590142986</v>
+      </c>
+      <c r="FN2" s="1" t="n">
+        <v>41905.09246254025</v>
       </c>
       <c r="FO2" s="1" t="n">
-        <v>7.024701666090977</v>
+        <v>7.092489757150096</v>
       </c>
       <c r="FP2" s="1" t="n">
-        <v>13.57815823144303</v>
+        <v>13.83650170118854</v>
       </c>
       <c r="FQ2" s="1" t="n">
-        <v>13.76539667861372</v>
+        <v>13.52044061844287</v>
       </c>
       <c r="FR2" s="1" t="n">
-        <v>34.36825657614774</v>
+        <v>34.44943207678151</v>
       </c>
       <c r="FS2" s="1" t="n">
-        <v>3252.074387212273</v>
+        <v>3255.493566629577</v>
       </c>
       <c r="FT2" t="n">
-        <v>6.7818229204602</v>
+        <v>6.786443914645855</v>
       </c>
       <c r="FU2" s="1" t="n">
-        <v>3063.027432629535</v>
+        <v>3052.174467014146</v>
       </c>
       <c r="FV2" s="1" t="n">
-        <v>855.1613518726423</v>
+        <v>854.308297656242</v>
       </c>
       <c r="FW2" s="1" t="n">
-        <v>20.86343894621884</v>
+        <v>21.22692831826694</v>
       </c>
       <c r="FX2" s="2" t="n">
-        <v>15.28802150719849</v>
+        <v>15.50771651327568</v>
       </c>
       <c r="FY2" s="2" t="n">
-        <v>36.15146045341733</v>
+        <v>36.73464483154262</v>
       </c>
       <c r="FZ2" s="2" t="n">
-        <v>11.90556901060386</v>
+        <v>12.98654517201299</v>
       </c>
       <c r="GA2" s="1" t="n">
-        <v>6.271293482506607</v>
+        <v>6.259535520648817</v>
       </c>
       <c r="GB2" s="1" t="n">
-        <v>151.7582244815</v>
+        <v>149.5241893965034</v>
       </c>
       <c r="GC2" s="1" t="n">
-        <v>239.3732284758779</v>
+        <v>238.163748643915</v>
       </c>
       <c r="GD2" s="1" t="n">
-        <v>34.36825657614773</v>
+        <v>34.4494320767815</v>
       </c>
       <c r="GE2" s="1" t="n">
-        <v>34.36825657614772</v>
+        <v>34.44943207678148</v>
       </c>
       <c r="GF2" s="1" t="n">
-        <v>2735.200698112158</v>
+        <v>2734.767989447653</v>
       </c>
       <c r="GG2" s="1" t="n">
         <v>-7.105427357601002e-15</v>
       </c>
-      <c r="GH2" t="n">
-        <v>7.105427357601002e-15</v>
+      <c r="GH2" s="2" t="n">
+        <v>2.131628207280301e-14</v>
       </c>
       <c r="GI2" s="1" t="n">
-        <v>12.65681015126646</v>
+        <v>8.221934482455424</v>
       </c>
       <c r="GJ2" s="1" t="n">
-        <v>-14.18304613779918</v>
+        <v>-18.03926279056452</v>
       </c>
       <c r="GK2" s="1" t="n">
-        <v>6.964951159088115</v>
+        <v>6.913430332119594</v>
       </c>
       <c r="GL2" s="1" t="n">
-        <v>85474.03623541899</v>
+        <v>85304.77045091939</v>
       </c>
       <c r="GM2" s="1" t="n">
-        <v>522.6174336242819</v>
-      </c>
-      <c r="GN2" s="1" t="n">
-        <v>4476.838485254198</v>
+        <v>520.4195952724123</v>
+      </c>
+      <c r="GN2" t="n">
+        <v>4459.849705375914</v>
       </c>
       <c r="GO2" s="1" t="n">
-        <v>109.6573505417168</v>
+        <v>110.2921527896275</v>
       </c>
       <c r="GP2" t="n">
-        <v>836.2776013788634</v>
+        <v>836.1205985386193</v>
       </c>
       <c r="GQ2" s="3" t="n">
-        <v>46124.95833333334</v>
+        <v>46126.95833333334</v>
       </c>
     </row>
     <row r="3">
@@ -2032,596 +2032,596 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>98.81869221048838</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>200000</v>
+        <v>97.3248155422659</v>
+      </c>
+      <c r="C3" t="n">
+        <v>196233.3870365402</v>
       </c>
       <c r="D3" t="n">
-        <v>85.348357196384</v>
+        <v>84.81794728597005</v>
       </c>
       <c r="E3" t="n">
-        <v>28.87847580567497</v>
+        <v>29.86438052079079</v>
       </c>
       <c r="F3" t="n">
-        <v>842.6576944817438</v>
+        <v>842.2453125593397</v>
       </c>
       <c r="G3" t="n">
-        <v>57155.90000596788</v>
+        <v>57165.86959201389</v>
       </c>
       <c r="H3" s="1" t="n">
-        <v>31.90140040328111</v>
+        <v>32.64923753484847</v>
       </c>
       <c r="I3" t="n">
-        <v>4414.93494547526</v>
+        <v>4418.076291232639</v>
       </c>
       <c r="J3" s="1" t="n">
-        <v>246.8352132934246</v>
+        <v>240.3394636809144</v>
       </c>
       <c r="K3" t="n">
-        <v>7360.421487901475</v>
+        <v>7357.398166232639</v>
       </c>
       <c r="L3" s="1" t="n">
-        <v>3884.509291467145</v>
+        <v>3862.161040377032</v>
       </c>
       <c r="M3" t="n">
-        <v>14.59539912144924</v>
+        <v>14.37677280690959</v>
       </c>
       <c r="N3" t="n">
-        <v>16.09203407296015</v>
+        <v>16.03911888285955</v>
       </c>
       <c r="O3" t="n">
-        <v>18.83281043479749</v>
+        <v>19.04962718826735</v>
       </c>
       <c r="P3" t="n">
-        <v>0.7767959800008982</v>
+        <v>0.5108625211175107</v>
       </c>
       <c r="Q3" t="n">
-        <v>18.06662320988469</v>
+        <v>18.11625065970433</v>
       </c>
       <c r="R3" t="n">
-        <v>290.0101920628007</v>
+        <v>290.505781224843</v>
       </c>
       <c r="S3" t="n">
-        <v>17.96496948108193</v>
+        <v>18.01872530053965</v>
       </c>
       <c r="T3" t="n">
-        <v>18.29332903910259</v>
+        <v>18.3489091825872</v>
       </c>
       <c r="U3" t="n">
-        <v>16.83967696133872</v>
+        <v>16.85512170690792</v>
       </c>
       <c r="V3" t="n">
-        <v>17.5247924803824</v>
+        <v>17.47341171865489</v>
       </c>
       <c r="W3" t="n">
-        <v>15.95296551798561</v>
+        <v>16.11508476008023</v>
       </c>
       <c r="X3" t="n">
-        <v>16.78773636655666</v>
+        <v>16.98475526444523</v>
       </c>
       <c r="Y3" t="n">
-        <v>15.98698359184501</v>
+        <v>15.54201876632454</v>
       </c>
       <c r="Z3" t="n">
-        <v>304.8101953804814</v>
+        <v>304.6532722517559</v>
       </c>
       <c r="AA3" t="n">
-        <v>1400.470064425485</v>
+        <v>1399.712373522052</v>
       </c>
       <c r="AB3" t="n">
-        <v>40.57847796105802</v>
+        <v>41.32790663383762</v>
       </c>
       <c r="AC3" t="n">
-        <v>800.0132895526766</v>
+        <v>799.9708947734933</v>
       </c>
       <c r="AD3" t="n">
-        <v>32.18420081938228</v>
+        <v>33.00818938960315</v>
       </c>
       <c r="AE3" s="1" t="n">
-        <v>79.2114513437613</v>
+        <v>77.3470733409081</v>
       </c>
       <c r="AF3" t="n">
-        <v>18.27885269588894</v>
+        <v>18.3017648129993</v>
       </c>
       <c r="AG3" t="n">
-        <v>198.8416915534126</v>
+        <v>197.8452721434326</v>
       </c>
       <c r="AH3" t="n">
-        <v>32.11438748448063</v>
+        <v>33.01682885789435</v>
       </c>
       <c r="AI3" t="n">
-        <v>34.93451950544255</v>
+        <v>35.97283846120372</v>
       </c>
       <c r="AJ3" t="n">
-        <v>203.1754389562441</v>
+        <v>201.4590200196819</v>
       </c>
       <c r="AK3" t="n">
-        <v>38.21450648444897</v>
+        <v>39.42238512068942</v>
       </c>
       <c r="AL3" t="n">
-        <v>449.9652374565553</v>
+        <v>452.3300378615192</v>
       </c>
       <c r="AM3" t="n">
-        <v>43.22966687433099</v>
+        <v>44.63835280195035</v>
       </c>
       <c r="AN3" t="n">
-        <v>989.5489964092047</v>
+        <v>988.9359199155318</v>
       </c>
       <c r="AO3" t="n">
-        <v>34.67384935208698</v>
+        <v>35.73468394642134</v>
       </c>
       <c r="AP3" t="n">
-        <v>1940.473365190136</v>
+        <v>1942.713186013357</v>
       </c>
       <c r="AQ3" t="n">
-        <v>242.3854250084702</v>
+        <v>242.1755184848817</v>
       </c>
       <c r="AR3" t="n">
-        <v>539.7055492122339</v>
+        <v>540.1758146174237</v>
       </c>
       <c r="AS3" t="n">
-        <v>1082.995338322184</v>
+        <v>1085.27512636813</v>
       </c>
       <c r="AT3" t="n">
-        <v>1911.107010262186</v>
+        <v>1917.684187624319</v>
       </c>
       <c r="AU3" t="n">
-        <v>99.35952136447766</v>
+        <v>100.4576666896562</v>
       </c>
       <c r="AV3" t="n">
-        <v>99.60142093287085</v>
+        <v>100.8734312561504</v>
       </c>
       <c r="AW3" t="n">
-        <v>105.9512477144461</v>
+        <v>107.2501222944425</v>
       </c>
       <c r="AX3" t="n">
-        <v>106.3554835841655</v>
+        <v>107.6587302940672</v>
       </c>
       <c r="AY3" t="n">
-        <v>95.76843548764639</v>
+        <v>96.69519790135796</v>
       </c>
       <c r="AZ3" t="n">
-        <v>8468.952514860366</v>
+        <v>8450.902524736193</v>
       </c>
       <c r="BA3" t="n">
-        <v>8239.654965294732</v>
+        <v>8218.649270587497</v>
       </c>
       <c r="BB3" t="n">
-        <v>8550.24224556817</v>
+        <v>8502.252428690592</v>
       </c>
       <c r="BC3" t="n">
-        <v>7867.709108988443</v>
+        <v>7822.475045628018</v>
       </c>
       <c r="BD3" t="n">
-        <v>7788.446044286091</v>
+        <v>7750.848289065891</v>
       </c>
       <c r="BE3" s="1" t="n">
-        <v>479.8300183924154</v>
+        <v>476.2905795729646</v>
       </c>
       <c r="BF3" t="n">
-        <v>-36.84912678429915</v>
+        <v>-36.84574792509388</v>
       </c>
       <c r="BG3" s="2" t="n">
-        <v>25.02623982984819</v>
+        <v>25.19682236645458</v>
       </c>
       <c r="BH3" t="n">
-        <v>179.6068804054969</v>
+        <v>180.7269279439286</v>
       </c>
       <c r="BI3" s="1" t="n">
-        <v>262.4781609082216</v>
+        <v>262.4028878990341</v>
       </c>
       <c r="BJ3" t="n">
-        <v>-20.56177921977318</v>
+        <v>-20.42557869526833</v>
       </c>
       <c r="BK3" t="n">
-        <v>171.689271281081</v>
+        <v>172.5678298490173</v>
       </c>
       <c r="BL3" t="n">
-        <v>532.8288359305047</v>
+        <v>521.7768965371132</v>
       </c>
       <c r="BM3" t="n">
-        <v>222.5874488777051</v>
+        <v>221.2991761258517</v>
       </c>
       <c r="BN3" t="n">
-        <v>48.65824039357815</v>
+        <v>49.48784729625582</v>
       </c>
       <c r="BO3" t="n">
-        <v>609.0547884843229</v>
+        <v>625.9043125014481</v>
       </c>
       <c r="BP3" t="n">
-        <v>1989.268917603081</v>
+        <v>2044.925754646833</v>
       </c>
       <c r="BQ3" t="n">
-        <v>103.6756565138099</v>
+        <v>105.014509473473</v>
       </c>
       <c r="BR3" t="n">
-        <v>226.7164183246115</v>
+        <v>229.9418141614595</v>
       </c>
       <c r="BS3" t="n">
-        <v>165.9412706192992</v>
+        <v>167.563452187068</v>
       </c>
       <c r="BT3" t="n">
-        <v>87.61500399437786</v>
+        <v>88.63955924741153</v>
       </c>
       <c r="BU3" t="n">
-        <v>4430.608328781358</v>
+        <v>4433.798892840635</v>
       </c>
       <c r="BV3" t="n">
-        <v>418.9206057179052</v>
+        <v>420.3838762862646</v>
       </c>
       <c r="BW3" s="1" t="n">
         <v>3724</v>
       </c>
       <c r="BX3" t="n">
-        <v>2117.867764687487</v>
+        <v>2116.918537219165</v>
       </c>
       <c r="BY3" t="n">
-        <v>15.97011746205296</v>
+        <v>16.20303567418958</v>
       </c>
       <c r="BZ3" t="n">
-        <v>52.99210852931461</v>
+        <v>53.25350461204947</v>
       </c>
       <c r="CA3" t="n">
-        <v>2479.953762400643</v>
+        <v>2490.674168523923</v>
       </c>
       <c r="CB3" t="n">
-        <v>1094.704710728958</v>
+        <v>1124.53018701425</v>
       </c>
       <c r="CC3" s="1" t="n">
-        <v>0.7864094656433048</v>
+        <v>0.784008503410605</v>
       </c>
       <c r="CD3" t="n">
-        <v>2.250554752675661</v>
+        <v>2.317626868429789</v>
       </c>
       <c r="CE3" t="n">
-        <v>-144.9966100436181</v>
+        <v>-144.9974314231062</v>
       </c>
       <c r="CF3" t="n">
-        <v>9.134824586844086</v>
+        <v>9.040561654281364</v>
       </c>
       <c r="CG3" t="n">
-        <v>-13.83017876866687</v>
+        <v>-13.7299829115497</v>
       </c>
       <c r="CH3" t="n">
-        <v>9.118757133841113</v>
+        <v>8.973377293491325</v>
       </c>
       <c r="CI3" t="n">
-        <v>-69.710179551971</v>
+        <v>-70.7415158625839</v>
       </c>
       <c r="CJ3" t="n">
-        <v>269.7793363841042</v>
+        <v>269.0368456613842</v>
       </c>
       <c r="CK3" t="n">
-        <v>2644.156546467249</v>
+        <v>2635.112429772635</v>
       </c>
       <c r="CL3" t="n">
-        <v>8.983371692111021</v>
+        <v>9.566313228303008</v>
       </c>
       <c r="CM3" t="n">
-        <v>77.77902387024814</v>
+        <v>76.94437624441434</v>
       </c>
       <c r="CN3" t="n">
-        <v>307.7769802244029</v>
+        <v>304.4441176520172</v>
       </c>
       <c r="CO3" t="n">
-        <v>3239.354945903857</v>
+        <v>3239.655051078771</v>
       </c>
       <c r="CP3" t="n">
-        <v>139.4160564635893</v>
+        <v>151.4108453169872</v>
       </c>
       <c r="CQ3" t="n">
-        <v>33.30007171630859</v>
+        <v>35.30004119873047</v>
       </c>
       <c r="CR3" t="n">
-        <v>175.6883113368979</v>
+        <v>175.4719457056262</v>
       </c>
       <c r="CS3" t="n">
-        <v>7.503603818242921</v>
+        <v>6.896210396122391</v>
       </c>
       <c r="CT3" t="n">
-        <v>5.812239416312256</v>
+        <v>5.311792281538858</v>
       </c>
       <c r="CU3" t="n">
-        <v>0.05301481755962111</v>
+        <v>0.03754002849996621</v>
       </c>
       <c r="CV3" t="n">
-        <v>2991.585474560653</v>
+        <v>2997.409859566566</v>
       </c>
       <c r="CW3" t="n">
-        <v>0.1210366375138174</v>
+        <v>0.09224786285573815</v>
       </c>
       <c r="CX3" t="n">
-        <v>17.26905897589323</v>
+        <v>18.11900051196469</v>
       </c>
       <c r="CY3" t="n">
-        <v>68.94845319439881</v>
+        <v>68.51558768270841</v>
       </c>
       <c r="CZ3" t="n">
         <v>105</v>
       </c>
       <c r="DA3" t="n">
-        <v>88.35028269541391</v>
+        <v>88.32133820475433</v>
       </c>
       <c r="DB3" t="n">
-        <v>72.57378432612231</v>
+        <v>72.49572429306056</v>
       </c>
       <c r="DC3" t="n">
-        <v>3.66395998052945</v>
+        <v>3.833675112531711</v>
       </c>
       <c r="DD3" t="n">
-        <v>17.76116411358734</v>
+        <v>13.81361400176535</v>
       </c>
       <c r="DE3" t="n">
-        <v>67.99499879211103</v>
+        <v>67.93809728353015</v>
       </c>
       <c r="DF3" t="n">
-        <v>3262.605488067773</v>
+        <v>3261.86282984533</v>
       </c>
       <c r="DG3" t="n">
-        <v>524.9563487206626</v>
+        <v>525.0989262197851</v>
       </c>
       <c r="DH3" t="n">
-        <v>-95.40830102543691</v>
+        <v>-95.74228136284748</v>
       </c>
       <c r="DI3" t="n">
-        <v>4.636369243435272</v>
+        <v>4.199992977743014</v>
       </c>
       <c r="DJ3" t="n">
-        <v>2989.750536133151</v>
+        <v>2989.267244112629</v>
       </c>
       <c r="DK3" t="n">
-        <v>-116.7022297241444</v>
+        <v>-117.9165558463937</v>
       </c>
       <c r="DL3" t="n">
-        <v>750.0585303068567</v>
+        <v>754.9545954521207</v>
       </c>
       <c r="DM3" t="n">
-        <v>53.45445653792587</v>
+        <v>54.24999025412212</v>
       </c>
       <c r="DN3" t="n">
-        <v>-56.50688991125233</v>
+        <v>-41.4344737703999</v>
       </c>
       <c r="DO3" s="1" t="n">
-        <v>25.08601612662113</v>
+        <v>25.09093072502913</v>
       </c>
       <c r="DP3" t="n">
-        <v>-98.92852320659505</v>
-      </c>
-      <c r="DQ3" s="2" t="n">
-        <v>19.5976352422147</v>
+        <v>-99.39330338806586</v>
+      </c>
+      <c r="DQ3" s="1" t="n">
+        <v>18.20111079591575</v>
       </c>
       <c r="DR3" s="1" t="n">
-        <v>57.15924189953441</v>
+        <v>56.2684357742443</v>
       </c>
       <c r="DS3" t="n">
-        <v>-74.06344771666863</v>
+        <v>-74.54844866170986</v>
       </c>
       <c r="DT3" t="n">
-        <v>33.2337575810471</v>
+        <v>30.69948667154742</v>
       </c>
       <c r="DU3" t="n">
-        <v>79.62947714839412</v>
+        <v>80.756324054592</v>
       </c>
       <c r="DV3" t="n">
-        <v>-53.86953281720486</v>
+        <v>-54.12040356920902</v>
       </c>
       <c r="DW3" t="n">
-        <v>825.6840684151401</v>
+        <v>818.9290604379709</v>
       </c>
       <c r="DX3" t="n">
-        <v>3073.196516326414</v>
+        <v>3072.122124083681</v>
       </c>
       <c r="DY3" s="1" t="n">
-        <v>44.34746219239543</v>
+        <v>43.92161983410615</v>
       </c>
       <c r="DZ3" s="1" t="n">
         <v>7613</v>
       </c>
       <c r="EA3" t="n">
-        <v>11.15814744000261</v>
+        <v>11.61825760009534</v>
       </c>
       <c r="EB3" t="n">
-        <v>48.34009790449397</v>
+        <v>49.55690453660036</v>
       </c>
       <c r="EC3" t="n">
-        <v>1871.478120039137</v>
+        <v>1883.618344916694</v>
       </c>
       <c r="ED3" s="1" t="n">
-        <v>10424.95900717817</v>
+        <v>10327.72554970067</v>
       </c>
       <c r="EE3" t="n">
-        <v>0.8223883137106895</v>
-      </c>
-      <c r="EF3" s="1" t="n">
-        <v>130</v>
+        <v>0.8240583389997482</v>
+      </c>
+      <c r="EF3" t="n">
+        <v>126.452726754487</v>
       </c>
       <c r="EG3" t="n">
-        <v>95.98804975412475</v>
+        <v>95.97200523152152</v>
       </c>
       <c r="EH3" t="n">
-        <v>0.9459427649003515</v>
+        <v>0.9233596056824488</v>
       </c>
       <c r="EI3" t="n">
-        <v>97.6175555828557</v>
+        <v>97.63591734287353</v>
       </c>
       <c r="EJ3" t="n">
-        <v>0.9431872915084042</v>
+        <v>0.9114688517023549</v>
       </c>
       <c r="EK3" t="n">
-        <v>299.4201775347054</v>
+        <v>299.5135586775037</v>
       </c>
       <c r="EL3" s="1" t="n">
-        <v>41355.99576472906</v>
-      </c>
-      <c r="EM3" s="1" t="n">
-        <v>843.9186909486469</v>
+        <v>40893.33068277877</v>
+      </c>
+      <c r="EM3" s="2" t="n">
+        <v>842.4028557648205</v>
       </c>
       <c r="EN3" t="n">
-        <v>649.9187321924995</v>
+        <v>648.6757025004936</v>
       </c>
       <c r="EO3" t="n">
-        <v>50.33966254419578</v>
+        <v>52.58045898343432</v>
       </c>
       <c r="EP3" t="n">
-        <v>65.37802829695413</v>
+        <v>65.22768847430098</v>
       </c>
       <c r="EQ3" t="n">
-        <v>63.55928097471713</v>
+        <v>64.24428018058454</v>
       </c>
       <c r="ER3" t="n">
-        <v>0.2904927058694518</v>
+        <v>0.2918296852988182</v>
       </c>
       <c r="ES3" t="n">
-        <v>109.6573505417168</v>
+        <v>110.2921527896275</v>
       </c>
       <c r="ET3" t="n">
-        <v>78.16269866877332</v>
+        <v>79.82268863403179</v>
       </c>
       <c r="EU3" t="n">
-        <v>29.99961232125018</v>
-      </c>
-      <c r="EV3" s="1" t="n">
-        <v>428.7274674254168</v>
-      </c>
-      <c r="EW3" s="1" t="n">
-        <v>1320.42139031569</v>
-      </c>
-      <c r="EX3" s="1" t="n">
-        <v>5865.875935770235</v>
-      </c>
-      <c r="EY3" s="2" t="n">
-        <v>1.944566142542782</v>
+        <v>29.99832643704054</v>
+      </c>
+      <c r="EV3" t="n">
+        <v>424.1379562353861</v>
+      </c>
+      <c r="EW3" t="n">
+        <v>1301.51653599988</v>
+      </c>
+      <c r="EX3" t="n">
+        <v>5761.366241375794</v>
+      </c>
+      <c r="EY3" t="n">
+        <v>1.944692855491665</v>
       </c>
       <c r="EZ3" t="n">
-        <v>26.08518441139056</v>
-      </c>
-      <c r="FA3" s="1" t="n">
-        <v>1244.251839868847</v>
-      </c>
-      <c r="FB3" s="1" t="n">
-        <v>3.901216754087349</v>
+        <v>26.0723117842812</v>
+      </c>
+      <c r="FA3" t="n">
+        <v>1239.193944973814</v>
+      </c>
+      <c r="FB3" t="n">
+        <v>3.861328239384998</v>
       </c>
       <c r="FC3" t="n">
-        <v>98.10277213745483</v>
+        <v>98.16088491447424</v>
       </c>
       <c r="FD3" t="n">
-        <v>1.390217379490118</v>
+        <v>1.344008784731304</v>
       </c>
       <c r="FE3" t="n">
         <v>11</v>
       </c>
-      <c r="FF3" s="1" t="n">
-        <v>0.643231284525167</v>
+      <c r="FF3" s="2" t="n">
+        <v>0.6377372248823372</v>
       </c>
       <c r="FG3" s="1" t="n">
-        <v>70</v>
-      </c>
-      <c r="FH3" s="2" t="n">
-        <v>35</v>
+        <v>69.7806602820532</v>
+      </c>
+      <c r="FH3" s="1" t="n">
+        <v>35.56003457712296</v>
       </c>
       <c r="FI3" s="2" t="n">
-        <v>2.78441765148796</v>
+        <v>2.788329389607038</v>
       </c>
       <c r="FJ3" s="1" t="n">
-        <v>172326.8842718333</v>
-      </c>
-      <c r="FK3" t="n">
-        <v>5.848705965880382</v>
+        <v>170815.7513055115</v>
+      </c>
+      <c r="FK3" s="1" t="n">
+        <v>5.865151487426162</v>
       </c>
       <c r="FL3" s="1" t="n">
-        <v>126918.3617078792</v>
-      </c>
-      <c r="FM3" s="2" t="n">
-        <v>12.17513464703528</v>
-      </c>
-      <c r="FN3" t="n">
-        <v>43763.69143976998</v>
+        <v>125946.1872477848</v>
+      </c>
+      <c r="FM3" s="1" t="n">
+        <v>12.45139590142986</v>
+      </c>
+      <c r="FN3" s="1" t="n">
+        <v>41905.09246254025</v>
       </c>
       <c r="FO3" s="1" t="n">
-        <v>7.253995496701065</v>
+        <v>7.224868506877135</v>
       </c>
       <c r="FP3" s="1" t="n">
-        <v>13.80290401038611</v>
+        <v>14.04358986615955</v>
       </c>
       <c r="FQ3" s="1" t="n">
-        <v>13.76539667861412</v>
+        <v>13.52044061844329</v>
       </c>
       <c r="FR3" s="1" t="n">
-        <v>34.8222961857013</v>
+        <v>34.78889899147998</v>
       </c>
       <c r="FS3" s="1" t="n">
-        <v>3252.074387212273</v>
+        <v>3255.493566629577</v>
       </c>
       <c r="FT3" t="n">
-        <v>6.7818229204602</v>
+        <v>6.786443914645855</v>
       </c>
       <c r="FU3" s="1" t="n">
-        <v>3063.027432629541</v>
+        <v>3052.174467014163</v>
       </c>
       <c r="FV3" s="1" t="n">
-        <v>855.161351881243</v>
+        <v>854.3082976647223</v>
       </c>
       <c r="FW3" s="1" t="n">
-        <v>20.86343894621884</v>
+        <v>21.22692831826695</v>
       </c>
       <c r="FX3" s="2" t="n">
-        <v>15.28802150719808</v>
+        <v>15.50771651327469</v>
       </c>
       <c r="FY3" s="2" t="n">
-        <v>36.15146045341692</v>
+        <v>36.73464483154163</v>
       </c>
       <c r="FZ3" s="2" t="n">
-        <v>11.90556901060352</v>
+        <v>12.98654517201192</v>
       </c>
       <c r="GA3" s="1" t="n">
-        <v>6.271293482506679</v>
+        <v>6.259535520648985</v>
       </c>
       <c r="GB3" s="1" t="n">
-        <v>155.3695135846578</v>
+        <v>152.2039105166519</v>
       </c>
       <c r="GC3" s="1" t="n">
-        <v>242.9845175790356</v>
+        <v>240.8434697640634</v>
       </c>
       <c r="GD3" s="1" t="n">
-        <v>34.8222961857013</v>
+        <v>34.78889899147998</v>
       </c>
       <c r="GE3" s="1" t="n">
-        <v>34.82229618570129</v>
+        <v>34.78889899147997</v>
       </c>
       <c r="GF3" s="1" t="n">
-        <v>2736.155646719893</v>
+        <v>2735.487620477015</v>
       </c>
       <c r="GG3" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="GH3" t="n">
-        <v>7.105427357601002e-15</v>
+      <c r="GH3" s="2" t="n">
+        <v>1.4210854715202e-14</v>
       </c>
       <c r="GI3" s="1" t="n">
-        <v>16.26809925442413</v>
+        <v>10.90165560260391</v>
       </c>
       <c r="GJ3" s="1" t="n">
-        <v>-10.57175703464142</v>
+        <v>-15.35954167041615</v>
       </c>
       <c r="GK3" s="1" t="n">
-        <v>6.977843054439636</v>
+        <v>6.9229977592291</v>
       </c>
       <c r="GL3" s="1" t="n">
-        <v>86603.25095760853</v>
+        <v>86009.95522395942</v>
       </c>
       <c r="GM3" s="1" t="n">
-        <v>534.1671930648557</v>
-      </c>
-      <c r="GN3" s="1" t="n">
-        <v>4545.454545454545</v>
+        <v>525.104553279084</v>
+      </c>
+      <c r="GN3" t="n">
+        <v>4459.849705375914</v>
       </c>
       <c r="GO3" s="1" t="n">
-        <v>112.46131589867</v>
+        <v>110.6292260705203</v>
       </c>
       <c r="GP3" t="inlineStr"/>
       <c r="GQ3" s="3" t="n">
-        <v>46124.95833333334</v>
+        <v>46126.95833333334</v>
       </c>
     </row>
   </sheetData>

</xml_diff>